<commit_message>
Dashboard module changes done
</commit_message>
<xml_diff>
--- a/fixtures/TestData.xlsx
+++ b/fixtures/TestData.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Tharushi\OrangeHRM_Playwright\OrangeHRM_Playwright_Project\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F995CCA7-C464-4C00-A886-76645396489B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFCFBDB1-2CB7-4335-B82D-C2A7CB4313FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F42E241A-864D-4689-9D6F-62EEF7EECB94}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{F42E241A-864D-4689-9D6F-62EEF7EECB94}"/>
   </bookViews>
   <sheets>
     <sheet name="Widget" sheetId="1" r:id="rId1"/>
     <sheet name="Quick Launch" sheetId="2" r:id="rId2"/>
+    <sheet name="UrlPart" sheetId="3" r:id="rId3"/>
+    <sheet name="Menu Items" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Time at Work</t>
   </si>
@@ -68,6 +70,66 @@
   </si>
   <si>
     <t>My Timesheet</t>
+  </si>
+  <si>
+    <t>UrlPart</t>
+  </si>
+  <si>
+    <t>leave/assignLeave</t>
+  </si>
+  <si>
+    <t>time/viewMyTimesheet</t>
+  </si>
+  <si>
+    <t>leave/viewMyLeaveList</t>
+  </si>
+  <si>
+    <t>leave/applyLeave</t>
+  </si>
+  <si>
+    <t>time/viewEmployeeTimesheet</t>
+  </si>
+  <si>
+    <t>leave/viewLeaveList</t>
+  </si>
+  <si>
+    <t>Menu Items</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>PIM</t>
+  </si>
+  <si>
+    <t>Leave</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Recruitment</t>
+  </si>
+  <si>
+    <t>My Info</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Directory</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>Claim</t>
+  </si>
+  <si>
+    <t>Buzz</t>
   </si>
 </sst>
 </file>
@@ -475,7 +537,8 @@
   <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -515,5 +578,132 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B89D74-9A0D-4F6C-9149-F72F22F1A4A3}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{753582E8-8396-4904-8349-746247A64BEC}">
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>